<commit_message>
feat: v4 - Grid Pivot, 117m Power Law, Wind sin/cos, Imputer Removal (Public 0.6137)
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/752fb57b23291faf/문서/contest/wind_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_2B59D2BFD3E0DD524542D1F050D4C0366D91F7E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49525FC2-E7E9-4BF8-9DE9-EE6973174E0A}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD3C0D10E8562C8F050FA30F667B1FB90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D798728-48D7-4965-8454-F6EB4E954E50}"/>
   <bookViews>
-    <workbookView xWindow="8000" yWindow="4550" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8340" yWindow="4890" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Timestamp</t>
   </si>
@@ -67,6 +67,9 @@
     <t>베이스라인 모듈화 및 로거 연동 테스트</t>
   </si>
   <si>
+    <t>2026-07-22 22:32:01</t>
+  </si>
+  <si>
     <t>v2</t>
   </si>
   <si>
@@ -79,7 +82,28 @@
     <t>LightGBM 교체 / 100m 고도 바람 변수 및 풍향(Wind Direction) 피처 추가</t>
   </si>
   <si>
-    <t>2026-07-22 22:32:01</t>
+    <t>2026-07-23 00:47:32</t>
+  </si>
+  <si>
+    <t>v3</t>
+  </si>
+  <si>
+    <t>5-Fold CV 도입 / 달력 피처 + GFS (80m/100m) 합성 풍속, v^3, 풍향</t>
+  </si>
+  <si>
+    <t>5-Fold OOF 평가 / K-Fold 교차 검증 적용으로 오버피팅 없는 OOF 점수 산출</t>
+  </si>
+  <si>
+    <t>2026-07-23 01:17:00</t>
+  </si>
+  <si>
+    <t>v4</t>
+  </si>
+  <si>
+    <t>격자별 Pivot 피처 + GFS/LDAPS 117m 멱법칙 보정 풍속 + 풍향 sin/cos 변환(360도와 1도의 경계 불연속 문제 해결) + SimpleImputer 제거(LightGBM 결측치 자체학습)</t>
+  </si>
+  <si>
+    <t>5-Fold OOF 평가 / v4: 공간 피처 확장, 117m 허브고도 보정, 무한대(inf) -&gt; nan 변환 적용</t>
   </si>
 </sst>
 </file>
@@ -435,19 +459,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.4140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.58203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.4140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.4140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="65.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="66.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="80.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
@@ -516,10 +531,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3">
         <v>0.79930000000000001</v>
@@ -531,19 +546,83 @@
         <v>0.66300000000000003</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3">
         <v>42</v>
       </c>
       <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3">
+        <v>0.60208994459999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>0.68640000000000001</v>
+      </c>
+      <c r="D4">
+        <v>0.90200000000000002</v>
+      </c>
+      <c r="E4">
+        <v>0.4708</v>
+      </c>
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="I3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" s="1">
-        <v>0.60208994459999998</v>
+      <c r="G4">
+        <v>42</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4">
+        <v>0.60569102330000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5">
+        <v>0.68859999999999999</v>
+      </c>
+      <c r="D5">
+        <v>0.90259999999999996</v>
+      </c>
+      <c r="E5">
+        <v>0.47449999999999998</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5">
+        <v>42</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0.61370839420000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: v5 - Foehn index, Heat stagnation index, Time-series Ramp diff/rolling (Public 0.615171)
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/752fb57b23291faf/문서/contest/wind_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD3C0D10E8562C8F050FA30F667B1FB90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D798728-48D7-4965-8454-F6EB4E954E50}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_2B59D2BFD320D2423143C7F050C208F65C15F962" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76CCE0FE-A6AD-4EBF-B37A-BC33538E59CF}"/>
   <bookViews>
     <workbookView xWindow="8340" yWindow="4890" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>Timestamp</t>
   </si>
@@ -104,6 +104,18 @@
   </si>
   <si>
     <t>5-Fold OOF 평가 / v4: 공간 피처 확장, 117m 허브고도 보정, 무한대(inf) -&gt; nan 변환 적용</t>
+  </si>
+  <si>
+    <t>2026-07-23 01:46:47</t>
+  </si>
+  <si>
+    <t>v5</t>
+  </si>
+  <si>
+    <t>v4 피처 + 푄현상(높새바람) 지수 + 열돔/대기정체 지수 + 시계열 Ramp(Diff/Rolling) 변동성</t>
+  </si>
+  <si>
+    <t>5-Fold OOF 평가 / v5: 태백 특수 기상 현상(푄/열돔) 및 시계열 바람 변동성 반영</t>
   </si>
 </sst>
 </file>
@@ -459,10 +471,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="9" max="9" width="80.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
@@ -621,8 +634,40 @@
       <c r="I5" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <v>0.61370839420000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6">
+        <v>0.68799999999999994</v>
+      </c>
+      <c r="D6">
+        <v>0.90249999999999997</v>
+      </c>
+      <c r="E6">
+        <v>0.47360000000000002</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.61517095129999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
need to check before we proceed to v6
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/752fb57b23291faf/문서/contest/wind_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_2B59D2BFD320D2423143C7F050C208F65C15F962" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76CCE0FE-A6AD-4EBF-B37A-BC33538E59CF}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="11_2B59D2BFD320D2423143C7F050C208F65C15F962" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E45213F6-4CD7-43A9-ABAF-BCA1AB96F3FB}"/>
   <bookViews>
-    <workbookView xWindow="8340" yWindow="4890" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="150" yWindow="3910" windowWidth="36270" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
   <si>
     <t>Timestamp</t>
   </si>
@@ -28,15 +28,6 @@
     <t>Version</t>
   </si>
   <si>
-    <t>Total Score</t>
-  </si>
-  <si>
-    <t>1 - NMAE</t>
-  </si>
-  <si>
-    <t>FICR</t>
-  </si>
-  <si>
     <t>Model</t>
   </si>
   <si>
@@ -49,9 +40,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Public Score</t>
-  </si>
-  <si>
     <t>2026-07-22 22:06:44</t>
   </si>
   <si>
@@ -116,13 +104,45 @@
   </si>
   <si>
     <t>5-Fold OOF 평가 / v5: 태백 특수 기상 현상(푄/열돔) 및 시계열 바람 변동성 반영</t>
+  </si>
+  <si>
+    <t>Val_Total Score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Val_1 - NMAE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Val_FICR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Leaderboard_Score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Leaderboard_1-nMAE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Leaderboard_FiCR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8639447416	</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3402351475	</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,20 +158,32 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="8.25"/>
+      <color rgb="FF485465"/>
+      <name val="Noto Sans KR"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF485465"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
-      <scheme val="major"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -166,9 +198,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -184,6 +224,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,14 +515,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="17"/>
   <cols>
+    <col min="1" max="1" width="18.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.08203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.9140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.08203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.4140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="149.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="80.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.4140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.58203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -486,36 +540,42 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
       </c>
       <c r="C2">
         <v>0.7137</v>
@@ -527,27 +587,33 @@
         <v>0.51259999999999994</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G2">
         <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="I2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2">
         <v>0.5932059435</v>
       </c>
+      <c r="K2" s="2">
+        <v>0.86146538110000004</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.32494650590000002</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>0.79930000000000001</v>
@@ -559,27 +625,33 @@
         <v>0.66300000000000003</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G3">
         <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3">
+        <v>15</v>
+      </c>
+      <c r="J3" s="2">
         <v>0.60208994459999998</v>
       </c>
+      <c r="K3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>0.68640000000000001</v>
@@ -591,27 +663,33 @@
         <v>0.4708</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G4">
         <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4">
+        <v>19</v>
+      </c>
+      <c r="J4" s="2">
         <v>0.60569102330000002</v>
       </c>
+      <c r="K4" s="2">
+        <v>0.86602318869999995</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.34535885789999998</v>
+      </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C5">
         <v>0.68859999999999999</v>
@@ -623,27 +701,34 @@
         <v>0.47449999999999998</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G5">
         <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5">
+        <v>23</v>
+      </c>
+      <c r="J5" s="2">
         <v>0.61370839420000001</v>
       </c>
+      <c r="K5" s="2">
+        <v>0.87077697679999999</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0.35663981150000001</v>
+      </c>
+      <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C6">
         <v>0.68799999999999994</v>
@@ -655,20 +740,27 @@
         <v>0.47360000000000002</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G6">
         <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J6" s="1">
+        <v>27</v>
+      </c>
+      <c r="J6" s="2">
         <v>0.61517095129999999</v>
       </c>
+      <c r="K6" s="3">
+        <v>0.8708219358</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0.35951996679999998</v>
+      </c>
+      <c r="M6" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>